<commit_message>
Guardar antes de hacer pull
</commit_message>
<xml_diff>
--- a/DocumentacionAuxiliar/FuentesUtilizadas.xlsx
+++ b/DocumentacionAuxiliar/FuentesUtilizadas.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jorge\Documents\Trabajo-Profesional\Javeriana\DocumentacionAuxiliar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3625E063-FE64-4AA1-A6A8-E19C26E2340D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E64504B8-04C5-4BD9-B8E2-1D14970984BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="59">
   <si>
     <t>Referencia</t>
   </si>
@@ -67,14 +68,158 @@
   </si>
   <si>
     <t>https://www.dane.gov.co/files/icer/2005/meta/t1.pdf?utm_source=chatgpt.com</t>
+  </si>
+  <si>
+    <t>Premium Wage Lit</t>
+  </si>
+  <si>
+    <t>Pais</t>
+  </si>
+  <si>
+    <t>Efecto cuantificado</t>
+  </si>
+  <si>
+    <t>Fuente</t>
+  </si>
+  <si>
+    <t>Peru</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	
+64% de premio en establecimientos grandes (&gt;200 empleados) frente a microempresas (2-5 empleados), tras controlar por educación y experiencia</t>
+  </si>
+  <si>
+    <t>Anderson (1997) pag6</t>
+  </si>
+  <si>
+    <t>Colombia</t>
+  </si>
+  <si>
+    <t>26.8% para directivos, 10% para profesionales y 8% para obreros en empresas grandes (&gt;200) frente al promedio nacional</t>
+  </si>
+  <si>
+    <t>Melo, Ramirez, Itagui (2012)</t>
+  </si>
+  <si>
+    <t>Estados unidos</t>
+  </si>
+  <si>
+    <t>35% de premio en empresas con 500 o más empleados en comparación con aquellas de menos de 500</t>
+  </si>
+  <si>
+    <t>Brown (1990)</t>
+  </si>
+  <si>
+    <t>Japon</t>
+  </si>
+  <si>
+    <t>Ratio salarial de 1.68 (las empresas de más de 1,000 empleados pagan un 68% más que las de 10-99 empleados)</t>
+  </si>
+  <si>
+    <t>Handbook Cap33</t>
+  </si>
+  <si>
+    <t>Nigeria</t>
+  </si>
+  <si>
+    <t>78.5% de premio (condicionado a capital humano) o más del 100% (uncondicionado) en firmas de 100+ empleados</t>
+  </si>
+  <si>
+    <t>Reed y Tran (2019)</t>
+  </si>
+  <si>
+    <t>Comoros</t>
+  </si>
+  <si>
+    <t>62.1% de premio condicionado o 73% uncondicionado en firmas grandes</t>
+  </si>
+  <si>
+    <t>Camerun</t>
+  </si>
+  <si>
+    <t>55.2% de premio salarial en firmas de 100+ empleados tras controles Mincerianos</t>
+  </si>
+  <si>
+    <t>42% de mayores ingresos en establecimientos de más de 500 empleados frente a los de 10-99 empleados</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anderson (1997) </t>
+  </si>
+  <si>
+    <t>Malasia</t>
+  </si>
+  <si>
+    <t>Los trabajadores en empresas de 1-9 empleados ganan un 32% menos que en empresas más grandes</t>
+  </si>
+  <si>
+    <t>Alemania</t>
+  </si>
+  <si>
+    <t>11% de premio salarial en firmas de gran escala (&gt;500 empleados</t>
+  </si>
+  <si>
+    <t>Lehmer, Moller (2006)</t>
+  </si>
+  <si>
+    <t>Suiza</t>
+  </si>
+  <si>
+    <t>3% de premio en firmas con más de 100 trabajadores frente a microempresas de menos de 5</t>
+  </si>
+  <si>
+    <t>Winter (1999)</t>
+  </si>
+  <si>
+    <t>Mexico</t>
+  </si>
+  <si>
+    <t>11.7% de premio condicionado en firmas de 100+ empleados</t>
+  </si>
+  <si>
+    <t>Chile</t>
+  </si>
+  <si>
+    <t>7.6% de premio salarial en firmas grandes tras controlar por características del trabajador</t>
+  </si>
+  <si>
+    <t>11.8% de premio condicionado en firmas de 100+ empleados</t>
+  </si>
+  <si>
+    <t>Paraguay</t>
+  </si>
+  <si>
+    <t>Zimbabue</t>
+  </si>
+  <si>
+    <t>Efecto reportado como significativamente mayor que el encontrado en Perú</t>
+  </si>
+  <si>
+    <t>Velenchik (1997)</t>
+  </si>
+  <si>
+    <t>32 Países (Bajo/Medio Ingreso)</t>
+  </si>
+  <si>
+    <t>Promedio de 34% (uncondicionado) y 15-18% (tras controlar por educación, experiencia y beneficios no pecuniarios)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -90,7 +235,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -98,14 +243,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -453,4 +616,216 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D4AF063-9829-4982-B7DA-666B5C880710}">
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="22.77734375" customWidth="1"/>
+    <col min="2" max="2" width="88.5546875" customWidth="1"/>
+    <col min="3" max="3" width="39.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+    </row>
+    <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" s="1" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" s="1" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" s="1" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" s="1" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" s="1" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>